<commit_message>
Atualiza monitoramento de voos
</commit_message>
<xml_diff>
--- a/docs/monitoramento_voos.xlsx
+++ b/docs/monitoramento_voos.xlsx
@@ -41,7 +41,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N7"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -347,6 +347,222 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:26:28+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>dfea699576d8a79f</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Azul / Gol</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-12-29T17:55:00</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-12-29T20:25:00</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>PT2H30M</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2027-01-06T15:40:00</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2027-01-07T01:30:00</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>PT9H50M</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2156</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>BRL</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>nao</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:26:28+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ee43f45f11b6eb57</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-12-29T17:55:00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-12-29T20:25:00</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>PT2H30M</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2027-01-06T09:30:00</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2027-01-06T12:10:00</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>PT2H40M</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2491</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>BRL</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>nao</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-26T22:26:28+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>48d1dbdd15a73ba6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-12-29T17:55:00</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-12-29T20:25:00</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>PT2H30M</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2027-01-06T22:40:00</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2027-01-07T01:20:00</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>PT2H40M</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2491</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>BRL</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>nao</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -403,7 +619,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-26T20:22:15+00:00</t>
+          <t>2026-07-26T22:26:28+00:00</t>
         </is>
       </c>
     </row>
@@ -415,7 +631,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
     </row>

</xml_diff>